<commit_message>
Made BPT diagrams and T_e plots for the LzLCS sample, as well as derived T_e and abundance errors for LzLCS.
</commit_message>
<xml_diff>
--- a/LzLCS/Final_LYC_EMISSION_LINES_David.xlsx
+++ b/LzLCS/Final_LYC_EMISSION_LINES_David.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10913"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ziboney/Library/CloudStorage/Dropbox/SH_student_2026/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0013ccd3bb406478/Senior Honours Project/LzLCS/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97554FB9-6B97-F84E-94BB-7CB8CBD96F7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11660" yWindow="500" windowWidth="27240" windowHeight="16440" xr2:uid="{BAAEC4FA-6A67-B54E-BD27-18D77EB399BD}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{BAAEC4FA-6A67-B54E-BD27-18D77EB399BD}"/>
   </bookViews>
   <sheets>
     <sheet name="Fluxes" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -659,9 +659,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0E4F732F-A22E-4C48-BED2-57CE41C5D682}">
   <dimension ref="A1:AY28"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="27.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="27.83203125" defaultRowHeight="16" x14ac:dyDescent="0.4"/>
   <sheetData>
-    <row r="1" spans="1:51" s="1" customFormat="1" ht="19" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:51" s="1" customFormat="1" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>27</v>
       </c>
@@ -816,7 +816,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="2" spans="1:51" s="1" customFormat="1" ht="19" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:51" s="1" customFormat="1" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A2" s="1" t="s">
         <v>76</v>
       </c>
@@ -973,7 +973,7 @@
         <v>0.13028834457097555</v>
       </c>
     </row>
-    <row r="3" spans="1:51" s="1" customFormat="1" ht="19" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:51" s="1" customFormat="1" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A3" s="1" t="s">
         <v>0</v>
       </c>
@@ -1128,7 +1128,7 @@
         <v>0.42505657000000002</v>
       </c>
     </row>
-    <row r="4" spans="1:51" s="1" customFormat="1" ht="19" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:51" s="1" customFormat="1" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A4" s="1" t="s">
         <v>1</v>
       </c>
@@ -1283,7 +1283,7 @@
         <v>0.43009624000000002</v>
       </c>
     </row>
-    <row r="5" spans="1:51" s="1" customFormat="1" ht="19" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:51" s="1" customFormat="1" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A5" s="1" t="s">
         <v>2</v>
       </c>
@@ -1438,7 +1438,7 @@
         <v>0.30524857</v>
       </c>
     </row>
-    <row r="6" spans="1:51" s="1" customFormat="1" ht="19" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:51" s="1" customFormat="1" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A6" s="1" t="s">
         <v>3</v>
       </c>
@@ -1593,7 +1593,7 @@
         <v>0.38292367999999999</v>
       </c>
     </row>
-    <row r="7" spans="1:51" s="1" customFormat="1" ht="19" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:51" s="1" customFormat="1" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A7" s="1" t="s">
         <v>4</v>
       </c>
@@ -1748,7 +1748,7 @@
         <v>0.42733784000000002</v>
       </c>
     </row>
-    <row r="8" spans="1:51" s="1" customFormat="1" ht="19" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:51" s="1" customFormat="1" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A8" s="1" t="s">
         <v>5</v>
       </c>
@@ -1903,7 +1903,7 @@
         <v>0.35689510000000002</v>
       </c>
     </row>
-    <row r="9" spans="1:51" s="1" customFormat="1" ht="19" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:51" s="1" customFormat="1" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A9" s="1" t="s">
         <v>6</v>
       </c>
@@ -2058,7 +2058,7 @@
         <v>0.42419876000000001</v>
       </c>
     </row>
-    <row r="10" spans="1:51" s="1" customFormat="1" ht="19" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:51" s="1" customFormat="1" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A10" s="1" t="s">
         <v>7</v>
       </c>
@@ -2213,7 +2213,7 @@
         <v>0.42650956000000001</v>
       </c>
     </row>
-    <row r="11" spans="1:51" s="1" customFormat="1" ht="19" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:51" s="1" customFormat="1" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A11" s="1" t="s">
         <v>8</v>
       </c>
@@ -2368,7 +2368,7 @@
         <v>0.42798868000000001</v>
       </c>
     </row>
-    <row r="12" spans="1:51" s="1" customFormat="1" ht="19" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:51" s="1" customFormat="1" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A12" s="1" t="s">
         <v>9</v>
       </c>
@@ -2523,7 +2523,7 @@
         <v>0.41854342999999999</v>
       </c>
     </row>
-    <row r="13" spans="1:51" s="1" customFormat="1" ht="19" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:51" s="1" customFormat="1" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A13" s="1" t="s">
         <v>10</v>
       </c>
@@ -2678,7 +2678,7 @@
         <v>0.42282650999999999</v>
       </c>
     </row>
-    <row r="14" spans="1:51" s="1" customFormat="1" ht="19" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:51" s="1" customFormat="1" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A14" s="1" t="s">
         <v>11</v>
       </c>
@@ -2833,7 +2833,7 @@
         <v>0.42947417999999998</v>
       </c>
     </row>
-    <row r="15" spans="1:51" s="1" customFormat="1" ht="19" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:51" s="1" customFormat="1" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A15" s="1" t="s">
         <v>12</v>
       </c>
@@ -2988,7 +2988,7 @@
         <v>0.41102362999999997</v>
       </c>
     </row>
-    <row r="16" spans="1:51" s="1" customFormat="1" ht="19" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:51" s="1" customFormat="1" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A16" s="1" t="s">
         <v>13</v>
       </c>
@@ -3143,7 +3143,7 @@
         <v>0.38256230000000002</v>
       </c>
     </row>
-    <row r="17" spans="1:51" s="1" customFormat="1" ht="19" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:51" s="1" customFormat="1" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A17" s="1" t="s">
         <v>14</v>
       </c>
@@ -3298,7 +3298,7 @@
         <v>0.42275056</v>
       </c>
     </row>
-    <row r="18" spans="1:51" s="1" customFormat="1" ht="19" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:51" s="1" customFormat="1" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A18" s="1" t="s">
         <v>15</v>
       </c>
@@ -3453,7 +3453,7 @@
         <v>0.43311431</v>
       </c>
     </row>
-    <row r="19" spans="1:51" s="1" customFormat="1" ht="19" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:51" s="1" customFormat="1" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A19" s="1" t="s">
         <v>16</v>
       </c>
@@ -3608,7 +3608,7 @@
         <v>0.43056875999999999</v>
       </c>
     </row>
-    <row r="20" spans="1:51" s="1" customFormat="1" ht="19" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:51" s="1" customFormat="1" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A20" s="1" t="s">
         <v>17</v>
       </c>
@@ -3763,7 +3763,7 @@
         <v>0.42808793000000001</v>
       </c>
     </row>
-    <row r="21" spans="1:51" s="1" customFormat="1" ht="19" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:51" s="1" customFormat="1" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A21" s="1" t="s">
         <v>18</v>
       </c>
@@ -3918,7 +3918,7 @@
         <v>0.42784857999999998</v>
       </c>
     </row>
-    <row r="22" spans="1:51" s="1" customFormat="1" ht="19" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:51" s="1" customFormat="1" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A22" s="1" t="s">
         <v>19</v>
       </c>
@@ -4073,7 +4073,7 @@
         <v>0.42953973000000001</v>
       </c>
     </row>
-    <row r="23" spans="1:51" s="1" customFormat="1" ht="19" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:51" s="1" customFormat="1" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A23" s="1" t="s">
         <v>20</v>
       </c>
@@ -4228,7 +4228,7 @@
         <v>0.42525555999999998</v>
       </c>
     </row>
-    <row r="24" spans="1:51" s="1" customFormat="1" ht="19" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:51" s="1" customFormat="1" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A24" s="1" t="s">
         <v>21</v>
       </c>
@@ -4383,7 +4383,7 @@
         <v>0.43060832999999998</v>
       </c>
     </row>
-    <row r="25" spans="1:51" s="1" customFormat="1" ht="19" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:51" s="1" customFormat="1" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A25" s="1" t="s">
         <v>22</v>
       </c>
@@ -4538,7 +4538,7 @@
         <v>0.42883652999999999</v>
       </c>
     </row>
-    <row r="26" spans="1:51" s="1" customFormat="1" ht="19" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:51" s="1" customFormat="1" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A26" s="1" t="s">
         <v>23</v>
       </c>
@@ -4693,7 +4693,7 @@
         <v>0.42745431</v>
       </c>
     </row>
-    <row r="27" spans="1:51" s="1" customFormat="1" ht="19" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:51" s="1" customFormat="1" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A27" s="1" t="s">
         <v>24</v>
       </c>
@@ -4848,7 +4848,7 @@
         <v>0.42555646000000003</v>
       </c>
     </row>
-    <row r="28" spans="1:51" s="1" customFormat="1" ht="19" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:51" s="1" customFormat="1" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A28" s="1" t="s">
         <v>25</v>
       </c>

</xml_diff>